<commit_message>
Updated test data and val issues
</commit_message>
<xml_diff>
--- a/rules/CORE-000249/negative/01/data/unit-test-coreid-CG0032-negative.xlsx
+++ b/rules/CORE-000249/negative/01/data/unit-test-coreid-CG0032-negative.xlsx
@@ -37,7 +37,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -63,9 +63,22 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -79,6 +92,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -108,7 +139,7 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -116,6 +147,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -576,7 +610,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="4" t="str">
-        <v>lb.xpt</v>
+        <v>tv.xpt</v>
       </c>
       <c r="C4" s="4" t="str">
         <v>Record</v>
@@ -689,248 +723,248 @@
       <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="6" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="6" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="6" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="6" t="str">
         <v>Sponsor-Defined Identifier</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="6" t="str">
         <v>Lab Test or Examination Short Name</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="6" t="str">
         <v>Lab Test or Examination Name</v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="6" t="str">
         <v>Category for Lab Test</v>
       </c>
-      <c r="I2" s="5" t="str">
+      <c r="I2" s="6" t="str">
         <v>Result or Finding in Original Units</v>
       </c>
-      <c r="J2" s="5" t="str">
+      <c r="J2" s="6" t="str">
         <v>Original Units</v>
       </c>
-      <c r="K2" s="5" t="str">
+      <c r="K2" s="6" t="str">
         <v>Reference Range Lower Limit in Orig Unit</v>
       </c>
-      <c r="L2" s="5" t="str">
+      <c r="L2" s="6" t="str">
         <v>Reference Range Upper Limit in Orig Unit</v>
       </c>
-      <c r="M2" s="5" t="str">
+      <c r="M2" s="6" t="str">
         <v>Character Result/Finding in Std Format</v>
       </c>
-      <c r="N2" s="5" t="str">
+      <c r="N2" s="6" t="str">
         <v>Numeric Result/Finding in Standard Units</v>
       </c>
-      <c r="O2" s="5" t="str">
+      <c r="O2" s="6" t="str">
         <v>Standard Units</v>
       </c>
-      <c r="P2" s="5" t="str">
+      <c r="P2" s="6" t="str">
         <v>Reference Range Lower Limit-Std Units</v>
       </c>
-      <c r="Q2" s="5" t="str">
+      <c r="Q2" s="6" t="str">
         <v>Reference Range Upper Limit-Std Units</v>
       </c>
-      <c r="R2" s="5" t="str">
+      <c r="R2" s="6" t="str">
         <v>Reference Range Indicator</v>
       </c>
-      <c r="S2" s="5" t="str">
+      <c r="S2" s="6" t="str">
         <v>LOINC Code</v>
       </c>
-      <c r="T2" s="5" t="str">
+      <c r="T2" s="6" t="str">
         <v>Specimen Type</v>
       </c>
-      <c r="U2" s="5" t="str">
+      <c r="U2" s="6" t="str">
         <v>Baseline Flag</v>
       </c>
-      <c r="V2" s="5" t="str">
+      <c r="V2" s="6" t="str">
         <v>Epoch</v>
       </c>
-      <c r="W2" s="5" t="str">
+      <c r="W2" s="6" t="str">
         <v>Visit Number</v>
       </c>
-      <c r="X2" s="5" t="str">
+      <c r="X2" s="6" t="str">
         <v>Visit Name</v>
       </c>
-      <c r="Y2" s="5" t="str">
+      <c r="Y2" s="6" t="str">
         <v>Date/Time of Specimen Collection</v>
       </c>
-      <c r="Z2" s="5" t="str">
+      <c r="Z2" s="6" t="str">
         <v>Study Day of Specimen Collection</v>
       </c>
-      <c r="AA2" s="5" t="str">
+      <c r="AA2" s="6" t="str">
         <v>Planned Study Day of Visit</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="5" t="str">
+      <c r="A3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="E3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="K3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="L3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="M3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="N3" s="5" t="str">
+      <c r="E3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="K3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="L3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="M3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="N3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="O3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="P3" s="5" t="str">
+      <c r="O3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="P3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="Q3" s="5" t="str">
+      <c r="Q3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="R3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="S3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="T3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="U3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="V3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="W3" s="5" t="str">
+      <c r="R3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="S3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="T3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="U3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="V3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="W3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="X3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Y3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Z3" s="5" t="str">
+      <c r="X3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Y3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Z3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="AA3" s="5" t="str">
+      <c r="AA3" s="6" t="str">
         <v>Num</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
+      <c r="A4" s="6">
         <v>10</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="6">
         <v>2</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="6">
         <v>14</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="6">
         <v>8</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="6">
         <v>4</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="6">
         <v>8</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="6">
         <v>25</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="6">
         <v>18</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="6">
         <v>6</v>
       </c>
-      <c r="J4" s="5">
+      <c r="J4" s="6">
         <v>8</v>
       </c>
-      <c r="K4" s="5">
+      <c r="K4" s="6">
         <v>1</v>
       </c>
-      <c r="L4" s="5">
+      <c r="L4" s="6">
         <v>1</v>
       </c>
-      <c r="M4" s="5">
+      <c r="M4" s="6">
         <v>6</v>
       </c>
-      <c r="N4" s="5">
+      <c r="N4" s="6">
         <v>8</v>
       </c>
-      <c r="O4" s="5">
+      <c r="O4" s="6">
         <v>8</v>
       </c>
-      <c r="P4" s="5">
+      <c r="P4" s="6">
         <v>8</v>
       </c>
-      <c r="Q4" s="5">
+      <c r="Q4" s="6">
         <v>8</v>
       </c>
-      <c r="R4" s="5">
+      <c r="R4" s="6">
         <v>1</v>
       </c>
-      <c r="S4" s="5">
+      <c r="S4" s="6">
         <v>7</v>
       </c>
-      <c r="T4" s="5">
+      <c r="T4" s="6">
         <v>5</v>
       </c>
-      <c r="U4" s="5">
+      <c r="U4" s="6">
         <v>1</v>
       </c>
-      <c r="V4" s="5">
+      <c r="V4" s="6">
         <v>9</v>
       </c>
-      <c r="W4" s="5">
+      <c r="W4" s="6">
         <v>8</v>
       </c>
-      <c r="X4" s="5">
+      <c r="X4" s="6">
         <v>18</v>
       </c>
-      <c r="Y4" s="5">
+      <c r="Y4" s="6">
         <v>10</v>
       </c>
-      <c r="Z4" s="5">
+      <c r="Z4" s="6">
         <v>8</v>
       </c>
-      <c r="AA4" s="5">
+      <c r="AA4" s="6">
         <v>8</v>
       </c>
     </row>
@@ -1001,7 +1035,7 @@
       <c r="V5" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="W5" s="6">
+      <c r="W5" s="7">
         <v>100</v>
       </c>
       <c r="X5" s="4" t="str">
@@ -1013,7 +1047,7 @@
       <c r="Z5" s="4" t="str">
         <v>-14</v>
       </c>
-      <c r="AA5" s="6" t="str">
+      <c r="AA5" s="8" t="str">
         <v>-15</v>
       </c>
     </row>
@@ -1138,80 +1172,80 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="str">
+      <c r="A2" s="6" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="6" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="6" t="str">
         <v>Visit Number</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="6" t="str">
         <v>Visit Name</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="6" t="str">
         <v>Planned Study Day of Visit</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="6" t="str">
         <v>Planned Arm Code</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="6" t="str">
         <v>Visit Start Rule</v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="6" t="str">
         <v>Visit End Rule</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="5" t="str">
+      <c r="A3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="D3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="E3" s="5" t="str">
+      <c r="D3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="E3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="F3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="5" t="str">
+      <c r="F3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="6" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
+      <c r="A4" s="6">
         <v>10</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="6">
         <v>2</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="6">
         <v>8</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="6">
         <v>18</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="6">
         <v>8</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="6">
         <v>1</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="6">
         <v>61</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="6">
         <v>21</v>
       </c>
     </row>
@@ -1228,7 +1262,7 @@
       <c r="D5" s="4" t="str">
         <v>VISIT 1 (WEEK -2)</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="9">
         <v>-14</v>
       </c>
       <c r="F5" s="4" t="str">

</xml_diff>